<commit_message>
feat: habilitar alerta de cumpleaños en dashboard para todos los roles
</commit_message>
<xml_diff>
--- a/empleados importacion/LISTA DE PERSONAL.xlsx
+++ b/empleados importacion/LISTA DE PERSONAL.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sistemas\vacaciones\empleados importacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EBD4853-1D8F-499C-B5E8-B5AD38225214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D440CA06-399A-4099-8F5E-0B1D0D51342D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -23,9 +23,7 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
       </xcalcf:calcFeatures>
@@ -35,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="319">
   <si>
     <t>Num</t>
   </si>
@@ -788,6 +786,210 @@
   </si>
   <si>
     <t>Sunza</t>
+  </si>
+  <si>
+    <t>DCP01</t>
+  </si>
+  <si>
+    <t>Distribuidora Comercial Peninsular FYVS</t>
+  </si>
+  <si>
+    <t>Ana Odilia</t>
+  </si>
+  <si>
+    <t>De la Cruz</t>
+  </si>
+  <si>
+    <t>Auxiliar de Imagen</t>
+  </si>
+  <si>
+    <t>Gabriela Selene</t>
+  </si>
+  <si>
+    <t>Caballero</t>
+  </si>
+  <si>
+    <t>Narvaez</t>
+  </si>
+  <si>
+    <t>Gerente Supervisión a Sucursales</t>
+  </si>
+  <si>
+    <t>Salvador</t>
+  </si>
+  <si>
+    <t>Pérez</t>
+  </si>
+  <si>
+    <t>Carrasco</t>
+  </si>
+  <si>
+    <t>Gerente de Tecnologías de la Información</t>
+  </si>
+  <si>
+    <t>Juan Gabriel</t>
+  </si>
+  <si>
+    <t>Jimenez</t>
+  </si>
+  <si>
+    <t>Chulim</t>
+  </si>
+  <si>
+    <t>Coordinador de produccion</t>
+  </si>
+  <si>
+    <t>Lizbeth Rubi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puc </t>
+  </si>
+  <si>
+    <t>Asistente Operativo</t>
+  </si>
+  <si>
+    <t>Sonia Carolina</t>
+  </si>
+  <si>
+    <t>Acereto</t>
+  </si>
+  <si>
+    <t>Jose Luis</t>
+  </si>
+  <si>
+    <t>Chab</t>
+  </si>
+  <si>
+    <t>Mariela Estefania</t>
+  </si>
+  <si>
+    <t>Abrego</t>
+  </si>
+  <si>
+    <t>Alcantara</t>
+  </si>
+  <si>
+    <t>Coordinación Creativa</t>
+  </si>
+  <si>
+    <t>Martha Maria</t>
+  </si>
+  <si>
+    <t>Villamil</t>
+  </si>
+  <si>
+    <t>Itzel Daniela</t>
+  </si>
+  <si>
+    <t>Campos</t>
+  </si>
+  <si>
+    <t>Content Manager</t>
+  </si>
+  <si>
+    <t>IMB01</t>
+  </si>
+  <si>
+    <t>Admon Insumos MB</t>
+  </si>
+  <si>
+    <t>Victor Adrian</t>
+  </si>
+  <si>
+    <t>Carrillo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Miguel Angel </t>
+  </si>
+  <si>
+    <t>Piña</t>
+  </si>
+  <si>
+    <t>Julio Cesar</t>
+  </si>
+  <si>
+    <t>Lavalle</t>
+  </si>
+  <si>
+    <t>Loria</t>
+  </si>
+  <si>
+    <t>Eddie Oswaldo</t>
+  </si>
+  <si>
+    <t>Noh</t>
+  </si>
+  <si>
+    <t>Adriana de Jesus</t>
+  </si>
+  <si>
+    <t>Cuevas</t>
+  </si>
+  <si>
+    <t>Borges</t>
+  </si>
+  <si>
+    <t>Encargada de Taller de Chapa</t>
+  </si>
+  <si>
+    <t>FAUSTO EDUARDO</t>
+  </si>
+  <si>
+    <t>GARCIA</t>
+  </si>
+  <si>
+    <t>ARJONA</t>
+  </si>
+  <si>
+    <t>Maria Jesus</t>
+  </si>
+  <si>
+    <t>Mis</t>
+  </si>
+  <si>
+    <t>Coordinadora imagen</t>
+  </si>
+  <si>
+    <t>Espinosa</t>
+  </si>
+  <si>
+    <t>Gestora eCommerce</t>
+  </si>
+  <si>
+    <t>Maria Fernanda</t>
+  </si>
+  <si>
+    <t>Guerrero</t>
+  </si>
+  <si>
+    <t>Especialista en Compras</t>
+  </si>
+  <si>
+    <t>Cinthia Anilu</t>
+  </si>
+  <si>
+    <t>Comprador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Litzy Maricarmen </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Duran </t>
+  </si>
+  <si>
+    <t>Cardenas</t>
+  </si>
+  <si>
+    <t>Atención al Cliente</t>
+  </si>
+  <si>
+    <t>Dianely Guadalupe</t>
+  </si>
+  <si>
+    <t>Alcala</t>
+  </si>
+  <si>
+    <t>Coordinador de RH</t>
   </si>
 </sst>
 </file>
@@ -1124,7 +1326,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I84"/>
+  <dimension ref="A1:I108"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="1"/>
@@ -3573,6 +3775,700 @@
         <v>234</v>
       </c>
     </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A85" s="3">
+        <v>2</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="E85" s="4">
+        <v>45028</v>
+      </c>
+      <c r="F85" s="4">
+        <v>31436</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="H85" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="I85" s="1" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A86" s="3">
+        <v>3</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="E86" s="4">
+        <v>39717</v>
+      </c>
+      <c r="F86" s="4">
+        <v>29777</v>
+      </c>
+      <c r="G86" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="H86" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="I86" s="1" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A87" s="3">
+        <v>4</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="E87" s="4">
+        <v>39128</v>
+      </c>
+      <c r="F87" s="4">
+        <v>27361</v>
+      </c>
+      <c r="G87" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="H87" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="I87" s="1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A88" s="3">
+        <v>5</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="E88" s="4">
+        <v>42555</v>
+      </c>
+      <c r="F88" s="4">
+        <v>28196</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="H88" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="I88" s="1" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A89" s="3">
+        <v>6</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="D89" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E89" s="4">
+        <v>43656</v>
+      </c>
+      <c r="F89" s="4">
+        <v>32671</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="H89" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="I89" s="1" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A90" s="3">
+        <v>8</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E90" s="4">
+        <v>45425</v>
+      </c>
+      <c r="F90" s="4">
+        <v>38212</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="H90" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="I90" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A91" s="3">
+        <v>11</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="E91" s="4">
+        <v>45943</v>
+      </c>
+      <c r="F91" s="4">
+        <v>35227</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="H91" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="I91" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A92" s="3">
+        <v>13</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="E92" s="4">
+        <v>46041</v>
+      </c>
+      <c r="F92" s="4">
+        <v>36887</v>
+      </c>
+      <c r="G92" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="H92" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="I92" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A93" s="3">
+        <v>14</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E93" s="4">
+        <v>46104</v>
+      </c>
+      <c r="F93" s="4">
+        <v>36659</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="H93" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="I93" s="1" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A94" s="3">
+        <v>15</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D94" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="E94" s="4">
+        <v>46162</v>
+      </c>
+      <c r="F94" s="4">
+        <v>37210</v>
+      </c>
+      <c r="G94" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="H94" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="I94" s="1" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A95" s="3">
+        <v>4</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E95" s="4">
+        <v>41183</v>
+      </c>
+      <c r="F95" s="4">
+        <v>28018</v>
+      </c>
+      <c r="G95" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H95" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="I95" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A96" s="3">
+        <v>8</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="D96" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E96" s="4">
+        <v>42402</v>
+      </c>
+      <c r="F96" s="4">
+        <v>33147</v>
+      </c>
+      <c r="G96" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H96" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="I96" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A97" s="3">
+        <v>9</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="D97" s="1"/>
+      <c r="E97" s="4">
+        <v>43165</v>
+      </c>
+      <c r="F97" s="4">
+        <v>28398</v>
+      </c>
+      <c r="G97" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H97" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="I97" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A98" s="3">
+        <v>10</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="D98" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="E98" s="4">
+        <v>38573</v>
+      </c>
+      <c r="F98" s="4">
+        <v>28296</v>
+      </c>
+      <c r="G98" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H98" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="I98" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A99" s="3">
+        <v>14</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D99" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="E99" s="4">
+        <v>42479</v>
+      </c>
+      <c r="F99" s="4">
+        <v>32247</v>
+      </c>
+      <c r="G99" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H99" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="I99" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A100" s="3">
+        <v>20</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="D100" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E100" s="4">
+        <v>42885</v>
+      </c>
+      <c r="F100" s="4">
+        <v>30123</v>
+      </c>
+      <c r="G100" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H100" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="I100" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A101" s="3">
+        <v>35</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="D101" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="E101" s="4">
+        <v>43662</v>
+      </c>
+      <c r="F101" s="4">
+        <v>31188</v>
+      </c>
+      <c r="G101" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H101" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="I101" s="1" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A102" s="3">
+        <v>58</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="D102" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="E102" s="4">
+        <v>44788</v>
+      </c>
+      <c r="F102" s="4">
+        <v>34963</v>
+      </c>
+      <c r="G102" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H102" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="I102" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A103" s="3">
+        <v>67</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D103" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="E103" s="4">
+        <v>39739</v>
+      </c>
+      <c r="F103" s="4">
+        <v>31993</v>
+      </c>
+      <c r="G103" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H103" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="I103" s="1" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A104" s="3">
+        <v>71</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="D104" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="E104" s="4">
+        <v>43206</v>
+      </c>
+      <c r="F104" s="4">
+        <v>34601</v>
+      </c>
+      <c r="G104" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H104" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="I104" s="1" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A105" s="3">
+        <v>73</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="D105" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="E105" s="4">
+        <v>43880</v>
+      </c>
+      <c r="F105" s="4">
+        <v>35739</v>
+      </c>
+      <c r="G105" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H105" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="I105" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A106" s="3">
+        <v>80</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D106" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E106" s="4">
+        <v>36778</v>
+      </c>
+      <c r="F106" s="4">
+        <v>29460</v>
+      </c>
+      <c r="G106" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H106" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="I106" s="1" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A107" s="3">
+        <v>86</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="D107" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="E107" s="4">
+        <v>45509</v>
+      </c>
+      <c r="F107" s="4">
+        <v>36796</v>
+      </c>
+      <c r="G107" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H107" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="I107" s="1" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A108" s="3">
+        <v>120</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="D108" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="E108" s="4">
+        <v>46042</v>
+      </c>
+      <c r="F108" s="4">
+        <v>34768</v>
+      </c>
+      <c r="G108" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H108" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="I108" s="1" t="s">
+        <v>318</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
refactor: make apple-touch-icon use dynamic logo path
</commit_message>
<xml_diff>
--- a/empleados importacion/LISTA DE PERSONAL.xlsx
+++ b/empleados importacion/LISTA DE PERSONAL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sistemas\vacaciones\empleados importacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D440CA06-399A-4099-8F5E-0B1D0D51342D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CF8F031-F2CE-4DC8-9C0F-42176DEAB4AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="770" uniqueCount="324">
   <si>
     <t>Num</t>
   </si>
@@ -990,13 +990,28 @@
   </si>
   <si>
     <t>Coordinador de RH</t>
+  </si>
+  <si>
+    <t>Carolina</t>
+  </si>
+  <si>
+    <t>Corrales</t>
+  </si>
+  <si>
+    <t>Editor de Video</t>
+  </si>
+  <si>
+    <t>MarÍa Jaqueline</t>
+  </si>
+  <si>
+    <t>Auxiliar de RH</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1012,8 +1027,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1024,6 +1053,47 @@
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
   </fills>
@@ -1326,7 +1396,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I108"/>
+  <dimension ref="A1:I128"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="1"/>
@@ -4469,6 +4539,586 @@
         <v>318</v>
       </c>
     </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A109" s="3">
+        <v>1</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D109" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="E109" s="4">
+        <v>35898</v>
+      </c>
+      <c r="F109" s="4">
+        <v>28064</v>
+      </c>
+      <c r="G109" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H109" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I109" s="1" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A110" s="3">
+        <v>7</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="D110" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="E110" s="4">
+        <v>38496</v>
+      </c>
+      <c r="F110" s="4">
+        <v>26983</v>
+      </c>
+      <c r="G110" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H110" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I110" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A111" s="3">
+        <v>81</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="D111" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="E111" s="4">
+        <v>40933</v>
+      </c>
+      <c r="F111" s="4">
+        <v>29584</v>
+      </c>
+      <c r="G111" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H111" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I111" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A112" s="3">
+        <v>185</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="D112" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="E112" s="4">
+        <v>42010</v>
+      </c>
+      <c r="F112" s="4">
+        <v>33181</v>
+      </c>
+      <c r="G112" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H112" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I112" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A113" s="3">
+        <v>271</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D113" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="E113" s="4">
+        <v>43088</v>
+      </c>
+      <c r="F113" s="4">
+        <v>32946</v>
+      </c>
+      <c r="G113" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H113" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I113" s="1" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A114" s="3">
+        <v>277</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="D114" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="E114" s="4">
+        <v>43203</v>
+      </c>
+      <c r="F114" s="4">
+        <v>34726</v>
+      </c>
+      <c r="G114" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H114" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I114" s="1" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A115" s="3">
+        <v>305</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="D115" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="E115" s="4">
+        <v>43684</v>
+      </c>
+      <c r="F115" s="4">
+        <v>35124</v>
+      </c>
+      <c r="G115" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H115" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I115" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A116" s="3">
+        <v>355</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="D116" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E116" s="4">
+        <v>45313</v>
+      </c>
+      <c r="F116" s="4">
+        <v>29354</v>
+      </c>
+      <c r="G116" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H116" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I116" s="1" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A117" s="3">
+        <v>363</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D117" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E117" s="4">
+        <v>45734</v>
+      </c>
+      <c r="F117" s="4">
+        <v>36198</v>
+      </c>
+      <c r="G117" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H117" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I117" s="1" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A118" s="3">
+        <v>365</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="D118" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="E118" s="4">
+        <v>45803</v>
+      </c>
+      <c r="F118" s="4">
+        <v>36794</v>
+      </c>
+      <c r="G118" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H118" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I118" s="1" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A119" s="3">
+        <v>366</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="C119" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="D119" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="E119" s="4">
+        <v>45880</v>
+      </c>
+      <c r="F119" s="4">
+        <v>33449</v>
+      </c>
+      <c r="G119" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H119" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I119" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A120" s="3">
+        <v>367</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="D120" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="E120" s="4">
+        <v>45901</v>
+      </c>
+      <c r="F120" s="4">
+        <v>33835</v>
+      </c>
+      <c r="G120" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H120" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I120" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A121" s="3">
+        <v>368</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C121" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D121" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E121" s="4">
+        <v>45615</v>
+      </c>
+      <c r="F121" s="4">
+        <v>28422</v>
+      </c>
+      <c r="G121" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H121" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I121" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A122" s="3">
+        <v>369</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D122" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E122" s="4">
+        <v>45617</v>
+      </c>
+      <c r="F122" s="4">
+        <v>38440</v>
+      </c>
+      <c r="G122" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H122" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I122" s="1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A123" s="3">
+        <v>370</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="D123" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E123" s="4">
+        <v>45979</v>
+      </c>
+      <c r="F123" s="4">
+        <v>39129</v>
+      </c>
+      <c r="G123" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H123" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I123" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A124" s="3">
+        <v>372</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C124" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="D124" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E124" s="4">
+        <v>46104</v>
+      </c>
+      <c r="F124" s="4">
+        <v>37417</v>
+      </c>
+      <c r="G124" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H124" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I124" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A125" s="3">
+        <v>373</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="D125" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="E125" s="4">
+        <v>46118</v>
+      </c>
+      <c r="F125" s="4">
+        <v>36433</v>
+      </c>
+      <c r="G125" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H125" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I125" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A126" s="3">
+        <v>374</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="C126" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D126" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="E126" s="4">
+        <v>46118</v>
+      </c>
+      <c r="F126" s="4">
+        <v>34926</v>
+      </c>
+      <c r="G126" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H126" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I126" s="1" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A127" s="3">
+        <v>375</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="C127" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="D127" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="E127" s="4">
+        <v>46181</v>
+      </c>
+      <c r="F127" s="4">
+        <v>36436</v>
+      </c>
+      <c r="G127" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H127" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I127" s="1" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A128" s="3">
+        <v>376</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="C128" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D128" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E128" s="4">
+        <v>46183</v>
+      </c>
+      <c r="F128" s="4">
+        <v>36079</v>
+      </c>
+      <c r="G128" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="H128" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I128" s="1" t="s">
+        <v>323</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>